<commit_message>
Regenerate fab packages for the sensor rename
BOM Comment/MPN now read TMR2615F-AAC-1.500-500 for U13-U23. Gerber and
drill diffs are plot-timestamp churn only; no copper changed. The
.kicad_pro hunk is kicad-cli bumping tuning_profiles.meta.version 0 -> 1.

DRC unchanged at 97 error-severity violations -- still not order-ready.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hw/TMR2615F_osu_pad/nextpcb/BOM-TMR2615F_osu_pad-nextpcb.xlsx
+++ b/hw/TMR2615F_osu_pad/nextpcb/BOM-TMR2615F_osu_pad-nextpcb.xlsx
@@ -1516,7 +1516,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMR2615x</t>
+          <t xml:space="preserve">TMR2615F-AAC-1.500-500</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMR2615F-AAC</t>
+          <t xml:space="preserve">TMR2615F-AAC-1.500-500</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">

</xml_diff>

<commit_message>
Regenerate fab packages for the pre-fab fixes
Both packages re-exported at 2026-08-04 04:05 from the corrected board.

Deltas that carry through to the portals: 32 -> 34 BOM lines and
150 -> 151 placements (U6 out, U25/U26 in), only TP1 now missing an LCSC
code where U2, U4 and TP1 were before, 644 -> 636 through vias, and 97 ->
96 error-severity DRC violations with 0 unconnected. Board outline,
stackup and layer set are unchanged.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hw/TMR2615F_osu_pad/nextpcb/BOM-TMR2615F_osu_pad-nextpcb.xlsx
+++ b/hw/TMR2615F_osu_pad/nextpcb/BOM-TMR2615F_osu_pad-nextpcb.xlsx
@@ -268,7 +268,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CL10B473KB8NNNC</t>
+          <t xml:space="preserve">CL10B332KB8NNNC</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -278,7 +278,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">47nF ±10% 50V Ceramic Capacitor X7R 0603</t>
+          <t xml:space="preserve">3.3nF ±10% 50V Ceramic Capacitor X7R 0603</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -288,7 +288,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CL10B473KB8NNNC</t>
+          <t xml:space="preserve">CL10B332KB8NNNC</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -298,7 +298,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">C1622</t>
+          <t xml:space="preserve">C1613</t>
         </is>
       </c>
     </row>
@@ -692,11 +692,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">R1,R2,R4,R5,R6,R9,R10,R26,R28</t>
+          <t xml:space="preserve">R1,R2,R4,R5,R6,R9,R10,R28</t>
         </is>
       </c>
       <c r="C15">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -788,15 +788,15 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">R8,R23,R24,R29,R30,R31,R32,R33,R34</t>
+          <t xml:space="preserve">R8,R12,R13,R15,R17,R18,R19,R20,R22,R29,R30,R31,R32,R33,R34</t>
         </is>
       </c>
       <c r="C17">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">0402WGF3300TCE</t>
+          <t xml:space="preserve">0402WGF5101TCE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">RES 330Ω ±1% 62.5mW 0402</t>
+          <t xml:space="preserve">5.1kΩ ±1% 62.5mW 0402 Thick Film Resistor</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">0402WGF3300TCE</t>
+          <t xml:space="preserve">0402WGF5101TCE</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t xml:space="preserve">C25104</t>
+          <t xml:space="preserve">C25905</t>
         </is>
       </c>
     </row>
@@ -884,15 +884,15 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">R12,R13,R15,R17,R18,R19,R20,R22</t>
+          <t xml:space="preserve">R23,R24</t>
         </is>
       </c>
       <c r="C19">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">0402WGF5101TCE</t>
+          <t xml:space="preserve">0402WGF3300TCE</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.1kΩ ±1% 62.5mW 0402 Thick Film Resistor</t>
+          <t xml:space="preserve">RES 330Ω ±1% 62.5mW 0402</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve">0402WGF5101TCE</t>
+          <t xml:space="preserve">0402WGF3300TCE</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t xml:space="preserve">C25905</t>
+          <t xml:space="preserve">C25104</t>
         </is>
       </c>
     </row>
@@ -980,25 +980,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW1,SW2</t>
+          <t xml:space="preserve">R26</t>
         </is>
       </c>
       <c r="C21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SKSGPAE010</t>
+          <t xml:space="preserve">0402WGF3301TCE</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW-SMD_SKSGAAE010</t>
+          <t xml:space="preserve">R_0402_1005Metric</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3.3kΩ ±1% 62.5mW 0402 Thick Film Resistor</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SKSGPAE010</t>
+          <t xml:space="preserve">0402WGF3301TCE</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t xml:space="preserve">C125045</t>
+          <t xml:space="preserve">C25890</t>
         </is>
       </c>
     </row>
@@ -1028,25 +1028,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW3,SW4,SW5,SW6,SW7,SW8</t>
+          <t xml:space="preserve">SW1,SW2</t>
         </is>
       </c>
       <c r="C22">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">CPG151101S11-16</t>
+          <t xml:space="preserve">SKSGPAE010</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMD_KEYBOARD-SW</t>
+          <t xml:space="preserve">SW-SMD_SKSGAAE010</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kailh-style MX hotswap socket (CPG151101S11-16)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">CPG151101S11-16</t>
+          <t xml:space="preserve">SKSGPAE010</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve">C41430893</t>
+          <t xml:space="preserve">C125045</t>
         </is>
       </c>
     </row>
@@ -1076,25 +1076,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP1,TP2,TP3,TP4,TP5,TP6,TP7,TP8,TP9,TP10,TP11,TP12,TP13,TP14,TP15,TP16,TP17,TP18,TP19,TP20,TP21,TP22</t>
+          <t xml:space="preserve">SW3,SW4,SW5,SW6,SW7,SW8</t>
         </is>
       </c>
       <c r="C23">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TestPoint</t>
+          <t xml:space="preserve">CPG151101S11-16</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TestPoint_Pad_D1.0mm</t>
+          <t xml:space="preserve">SMD_KEYBOARD-SW</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">test point</t>
+          <t xml:space="preserve">Kailh-style MX hotswap socket (CPG151101S11-16)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1104,17 +1104,17 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">CPG151101S11-16</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">LCSC</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">C41430893</t>
         </is>
       </c>
     </row>
@@ -1124,25 +1124,25 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">U1,U5,U6,U9</t>
+          <t xml:space="preserve">TP1,TP2,TP3,TP4,TP5,TP6,TP7,TP8,TP9,TP10,TP11,TP12,TP13,TP14,TP15,TP16,TP17,TP18,TP19,TP20,TP21,TP22</t>
         </is>
       </c>
       <c r="C24">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRV05-4A</t>
+          <t xml:space="preserve">TestPoint</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23-6</t>
+          <t xml:space="preserve">TestPoint_Pad_D1.0mm</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESD Protection Diodes with Low Clamping Voltage, SOT-23-6</t>
+          <t xml:space="preserve">test point</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRV05-4A</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCSC</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t xml:space="preserve">C20615829</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -1172,25 +1172,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">U2,U7</t>
+          <t xml:space="preserve">U1,U5,U9</t>
         </is>
       </c>
       <c r="C25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">LM66100DCK</t>
+          <t xml:space="preserve">SRV05-4A</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-363_SC-70-6</t>
+          <t xml:space="preserve">SOT-23-6</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ideal Diode With Input Polarity Protection 1.5 - 5.5V  Input Voltage, 1.5A Output Current, Ron 141 mOhm, SC-70-6</t>
+          <t xml:space="preserve">ESD Protection Diodes with Low Clamping Voltage, SOT-23-6</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1200,17 +1200,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">LM66100DCK</t>
+          <t xml:space="preserve">SRV05-4A</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">LCSC</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">C20615829</t>
         </is>
       </c>
     </row>
@@ -1220,25 +1220,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">U3</t>
+          <t xml:space="preserve">U2,U7</t>
         </is>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">AP22653W6-7</t>
+          <t xml:space="preserve">LM66100DCK</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23-6_L2.9-W1.6-P0.95-LS2.8-BR</t>
+          <t xml:space="preserve">SOT-363_SC-70-6</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">USB power switch / eFuse, 0.5-2.1A precision-adjustable current limit via R_ILIM, reverse-current blocking, soft-start, FLG fault flag, active-high EN — Diodes AP22653W6-7</t>
+          <t xml:space="preserve">Ideal Diode With Input Polarity Protection 1.5 - 5.5V  Input Voltage, 1.5A Output Current, Ron 141 mOhm, SC-70-6</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">AP22653W6-7</t>
+          <t xml:space="preserve">LM66100DCK</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2158037</t>
+          <t xml:space="preserve">C2869734</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">U4</t>
+          <t xml:space="preserve">U3</t>
         </is>
       </c>
       <c r="C27">
@@ -1276,37 +1276,37 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TPS7A4700</t>
+          <t xml:space="preserve">AP22653W6-7</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">VQFN-20_L5.0-W5.0-P0.65-TL-EP</t>
+          <t xml:space="preserve">SOT-23-6_L2.9-W1.6-P0.95-LS2.8-BR</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">USB power switch / eFuse, 0.5-2.1A precision-adjustable current limit via R_ILIM, reverse-current blocking, soft-start, FLG fault flag, active-high EN — Diodes AP22653W6-7</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texas Instruments</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TPS7A4700RGWT</t>
+          <t xml:space="preserve">AP22653W6-7</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">LCSC</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">C2158037</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">U8</t>
+          <t xml:space="preserve">U4</t>
         </is>
       </c>
       <c r="C28">
@@ -1324,27 +1324,27 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">XC6206P332MR</t>
+          <t xml:space="preserve">TPS7A4700</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23-3_L2.9-W1.6-P1.90-LS2.8-BR</t>
+          <t xml:space="preserve">VQFN-20_L5.0-W5.0-P0.65-TL-EP</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.3V 200mA 6V</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Texas Instruments</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">XC6206P332MR</t>
+          <t xml:space="preserve">TPS7A4700RGWT</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t xml:space="preserve">C5446</t>
+          <t xml:space="preserve">C28286</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">U10</t>
+          <t xml:space="preserve">U8</t>
         </is>
       </c>
       <c r="C29">
@@ -1372,17 +1372,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">AT32F405RBT7-7</t>
+          <t xml:space="preserve">XC6206P332MR</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">LQFP-64_L7.0-W7.0-P0.40-LS9.0-BL</t>
+          <t xml:space="preserve">SOT-23-3_L2.9-W1.6-P1.90-LS2.8-BR</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARM Cortex-M4F MCU, 216 MHz, 128KB Flash, 96+6KB SRAM, USB 2.0 HS+FS PHY, 1× 12-bit 2 MSPS ADC w/ 16-bit oversampling — Artery AT32F405RBT7-7</t>
+          <t xml:space="preserve">3.3V 200mA 6V</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">AT32F405RBT7-7</t>
+          <t xml:space="preserve">XC6206P332MR</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t xml:space="preserve">C47115472</t>
+          <t xml:space="preserve">C5446</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">U11</t>
+          <t xml:space="preserve">U10</t>
         </is>
       </c>
       <c r="C30">
@@ -1420,17 +1420,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMUX1574RSVR</t>
+          <t xml:space="preserve">AT32F405RBT7-7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">UQFN-16_L2.6-W1.8-P0.40-BL</t>
+          <t xml:space="preserve">LQFP-64_L7.0-W7.0-P0.40-LS9.0-BL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quad SPDT (4× 2:1) analog mux, 1.5-5.5V, 2Ω Ron, low charge injection (TI TMUX1574), UQFN-16 package</t>
+          <t xml:space="preserve">ARM Cortex-M4F MCU, 216 MHz, 128KB Flash, 96+6KB SRAM, USB 2.0 HS+FS PHY, 1× 12-bit 2 MSPS ADC w/ 16-bit oversampling — Artery AT32F405RBT7-7</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMUX1574RSVR</t>
+          <t xml:space="preserve">AT32F405RBT7-7</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2673120</t>
+          <t xml:space="preserve">C47115472</t>
         </is>
       </c>
     </row>
@@ -1460,25 +1460,25 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">U12,U14,U16,U18,U20,U22,U24</t>
+          <t xml:space="preserve">U11</t>
         </is>
       </c>
       <c r="C31">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">SK6812MINI-E</t>
+          <t xml:space="preserve">TMUX1574RSVR</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED-SMD_4P-L3.2-W2.8-LS5.9_SK6812MINI-E</t>
+          <t xml:space="preserve">UQFN-16_L2.6-W1.8-P0.40-BL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">SK6812MINI-E addressable RGB LED, 5V, 4-pin SMD reverse-mount</t>
+          <t xml:space="preserve">Quad SPDT (4× 2:1) analog mux, 1.5-5.5V, 2Ω Ron, low charge injection (TI TMUX1574), UQFN-16 package</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve">SK6812MINI-E</t>
+          <t xml:space="preserve">TMUX1574RSVR</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t xml:space="preserve">C5149201</t>
+          <t xml:space="preserve">C2673120</t>
         </is>
       </c>
     </row>
@@ -1508,35 +1508,35 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">U13,U15,U17,U19,U21,U23</t>
+          <t xml:space="preserve">U12,U14,U16,U18,U20,U22,U24</t>
         </is>
       </c>
       <c r="C32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMR2615F-AAC-1.500-500</t>
+          <t xml:space="preserve">SK6812MINI-E</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">DFN3L(1.6x1.6x0.5)</t>
+          <t xml:space="preserve">LED-SMD_4P-L3.2-W2.8-LS5.9_SK6812MINI-E</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low Power Large Range TMR Linear Magnetic Sens</t>
+          <t xml:space="preserve">SK6812MINI-E addressable RGB LED, 5V, 4-pin SMD reverse-mount</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">MultiDimension Technology (MDT)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMR2615F-AAC-1.500-500</t>
+          <t xml:space="preserve">SK6812MINI-E</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t xml:space="preserve">C9900212297</t>
+          <t xml:space="preserve">C5149201</t>
         </is>
       </c>
     </row>
@@ -1556,43 +1556,139 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t xml:space="preserve">U13,U15,U17,U19,U21,U23</t>
+        </is>
+      </c>
+      <c r="C33">
+        <v>6</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TMR2615F-AAC-1.500-500</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DFN3L(1.6x1.6x0.5)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low Power Large Range TMR Linear Magnetic Sens</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MultiDimension Technology (MDT)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TMR2615F-AAC-1.500-500</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LCSC</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C9900212297</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">U25,U26</t>
+        </is>
+      </c>
+      <c r="C34">
+        <v>2</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PESD5V0R1BSFYL</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SOD-962_L0.6-W0.3-BI</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bidirectional ESD, 5V VRWM, 0.15pF max line capacitance (TrEOS), IEC 61000-4-2 ±8kV contact, SOD-962/DSN0603-2</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PESD5V0R1BSFYL</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LCSC</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C461221</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t xml:space="preserve">X1</t>
         </is>
       </c>
-      <c r="C33">
+      <c r="C35">
         <v>1</v>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t xml:space="preserve">X322512MSB4SI</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t xml:space="preserve">X322512MSB4SI</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t xml:space="preserve">Crystal 12MHz ±10ppm 20pF SMD3225-4P</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
+      <c r="G35" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t xml:space="preserve">X322512MSB4SI</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LCSC</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LCSC</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t xml:space="preserve">C9002</t>
         </is>

</xml_diff>